<commit_message>
re-gen excel templates when update the data in DB
</commit_message>
<xml_diff>
--- a/backend/templates/template_antenna.xlsx
+++ b/backend/templates/template_antenna.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Antennas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Antennas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Antennas'!$A$1:$O$1</definedName>
@@ -17705,21 +17705,21 @@
   </sheetData>
   <autoFilter ref="A1:O1"/>
   <dataValidations count="5">
-    <dataValidation sqref="C2:C1001" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+    <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"x,"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1001" showErrorMessage="1" showInputMessage="1" allowBlank="1" errorTitle="Số cổng không hợp lệ" error="Phải là số nguyên 1 – 32" type="whole" operator="between">
+    <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Số cổng không hợp lệ" error="Phải là số nguyên 1 – 32" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>32</formula2>
     </dataValidation>
-    <dataValidation sqref="E2:E1001" showErrorMessage="1" showInputMessage="1" allowBlank="1" errorTitle="Số beam không hợp lệ" error="Phải là số nguyên 1 – 64" type="whole" operator="between">
+    <dataValidation sqref="E2:E1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Số beam không hợp lệ" error="Phải là số nguyên 1 – 64" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>64</formula2>
     </dataValidation>
-    <dataValidation sqref="B2:B1001" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"700,850,900,1800,2100,2600,3500,900-1800,900-2100,1800-2100,700-1800-2100,900-1800-2100,700-1800-2100-2600,3500-26000"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1001" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+    <dataValidation sqref="N2:N1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"4.3-10,7/16 DIN,N-Type,SMA,TNC,EIA 7/8""</formula1>
     </dataValidation>
   </dataValidations>
@@ -18299,11 +18299,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>